<commit_message>
Undo & re-auction workflow, flash cleanup fix, min-bid check
</commit_message>
<xml_diff>
--- a/2026 Auction List 75 players.xlsx
+++ b/2026 Auction List 75 players.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fount\Dropbox\ClaudeCoWork\Auction App Creation\C&amp;A Auction\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{01005647-FBEF-4F26-9079-9A07EF5EF323}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1B5E771-FE94-481A-BD29-C92993DD1760}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="11520" xr2:uid="{C5D6A754-9301-4B43-9C73-F98CF5D4264B}"/>
   </bookViews>
@@ -278,9 +278,6 @@
     <t>Bhayshul Tuten</t>
   </si>
   <si>
-    <t>Rank</t>
-  </si>
-  <si>
     <t>QB</t>
   </si>
   <si>
@@ -384,6 +381,9 @@
   </si>
   <si>
     <t>ADP</t>
+  </si>
+  <si>
+    <t>Auction#</t>
   </si>
 </sst>
 </file>
@@ -778,19 +778,19 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>79</v>
+        <v>114</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>113</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -798,7 +798,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>0</v>
@@ -815,7 +815,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>2</v>
@@ -832,7 +832,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>4</v>
@@ -849,7 +849,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>6</v>
@@ -866,7 +866,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>8</v>
@@ -883,7 +883,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>10</v>
@@ -900,7 +900,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>12</v>
@@ -917,7 +917,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>14</v>
@@ -934,7 +934,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C10" s="3" t="s">
         <v>16</v>
@@ -951,7 +951,7 @@
         <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>18</v>
@@ -968,7 +968,7 @@
         <v>11</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C12" s="3" t="s">
         <v>20</v>
@@ -985,7 +985,7 @@
         <v>12</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C13" s="3" t="s">
         <v>22</v>
@@ -1002,7 +1002,7 @@
         <v>13</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C14" s="3" t="s">
         <v>24</v>
@@ -1019,7 +1019,7 @@
         <v>14</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C15" s="3" t="s">
         <v>26</v>
@@ -1036,7 +1036,7 @@
         <v>15</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C16" s="3" t="s">
         <v>28</v>
@@ -1053,7 +1053,7 @@
         <v>16</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C17" s="3" t="s">
         <v>30</v>
@@ -1070,7 +1070,7 @@
         <v>17</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C18" s="3" t="s">
         <v>32</v>
@@ -1087,7 +1087,7 @@
         <v>18</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C19" s="3" t="s">
         <v>34</v>
@@ -1104,7 +1104,7 @@
         <v>19</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C20" s="3" t="s">
         <v>36</v>
@@ -1121,7 +1121,7 @@
         <v>20</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C21" s="3" t="s">
         <v>38</v>
@@ -1138,7 +1138,7 @@
         <v>21</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C22" s="3" t="s">
         <v>40</v>
@@ -1155,7 +1155,7 @@
         <v>22</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C23" s="3" t="s">
         <v>42</v>
@@ -1172,7 +1172,7 @@
         <v>23</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C24" s="3" t="s">
         <v>46</v>
@@ -1189,7 +1189,7 @@
         <v>24</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C25" s="3" t="s">
         <v>47</v>
@@ -1206,7 +1206,7 @@
         <v>25</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C26" s="3" t="s">
         <v>49</v>
@@ -1223,7 +1223,7 @@
         <v>26</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C27" s="3" t="s">
         <v>50</v>
@@ -1240,7 +1240,7 @@
         <v>27</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C28" s="3" t="s">
         <v>51</v>
@@ -1257,7 +1257,7 @@
         <v>28</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C29" s="3" t="s">
         <v>52</v>
@@ -1274,7 +1274,7 @@
         <v>29</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C30" s="3" t="s">
         <v>54</v>
@@ -1291,7 +1291,7 @@
         <v>30</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C31" s="3" t="s">
         <v>55</v>
@@ -1308,7 +1308,7 @@
         <v>31</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C32" s="3" t="s">
         <v>56</v>
@@ -1325,7 +1325,7 @@
         <v>32</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C33" s="3" t="s">
         <v>57</v>
@@ -1342,7 +1342,7 @@
         <v>33</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C34" s="3" t="s">
         <v>58</v>
@@ -1359,7 +1359,7 @@
         <v>34</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C35" s="3" t="s">
         <v>59</v>
@@ -1376,7 +1376,7 @@
         <v>35</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C36" s="3" t="s">
         <v>60</v>
@@ -1393,7 +1393,7 @@
         <v>36</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C37" s="3" t="s">
         <v>61</v>
@@ -1410,7 +1410,7 @@
         <v>37</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C38" s="3" t="s">
         <v>62</v>
@@ -1427,7 +1427,7 @@
         <v>38</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C39" s="3" t="s">
         <v>64</v>
@@ -1444,7 +1444,7 @@
         <v>39</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C40" s="3" t="s">
         <v>65</v>
@@ -1461,7 +1461,7 @@
         <v>40</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C41" s="3" t="s">
         <v>67</v>
@@ -1478,7 +1478,7 @@
         <v>41</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C42" s="3" t="s">
         <v>68</v>
@@ -1495,7 +1495,7 @@
         <v>42</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C43" s="3" t="s">
         <v>70</v>
@@ -1512,7 +1512,7 @@
         <v>43</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C44" s="3" t="s">
         <v>71</v>
@@ -1529,7 +1529,7 @@
         <v>44</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C45" s="3" t="s">
         <v>72</v>
@@ -1546,7 +1546,7 @@
         <v>45</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C46" s="3" t="s">
         <v>73</v>
@@ -1563,7 +1563,7 @@
         <v>46</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C47" s="3" t="s">
         <v>74</v>
@@ -1580,7 +1580,7 @@
         <v>47</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C48" s="3" t="s">
         <v>75</v>
@@ -1597,7 +1597,7 @@
         <v>48</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C49" s="3" t="s">
         <v>77</v>
@@ -1614,7 +1614,7 @@
         <v>49</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C50" s="3" t="s">
         <v>78</v>
@@ -1631,10 +1631,10 @@
         <v>50</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D51" s="4" t="s">
         <v>7</v>
@@ -1648,10 +1648,10 @@
         <v>51</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D52" s="4" t="s">
         <v>31</v>
@@ -1665,10 +1665,10 @@
         <v>52</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D53" s="4" t="s">
         <v>45</v>
@@ -1682,10 +1682,10 @@
         <v>53</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D54" s="4" t="s">
         <v>33</v>
@@ -1699,10 +1699,10 @@
         <v>54</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D55" s="4" t="s">
         <v>3</v>
@@ -1716,10 +1716,10 @@
         <v>55</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D56" s="4" t="s">
         <v>15</v>
@@ -1733,10 +1733,10 @@
         <v>56</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D57" s="4" t="s">
         <v>43</v>
@@ -1750,10 +1750,10 @@
         <v>57</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D58" s="4" t="s">
         <v>23</v>
@@ -1767,10 +1767,10 @@
         <v>58</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D59" s="4" t="s">
         <v>48</v>
@@ -1784,10 +1784,10 @@
         <v>59</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D60" s="4" t="s">
         <v>15</v>
@@ -1801,10 +1801,10 @@
         <v>60</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D61" s="4" t="s">
         <v>29</v>
@@ -1818,10 +1818,10 @@
         <v>61</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C62" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D62" s="4" t="s">
         <v>9</v>
@@ -1835,10 +1835,10 @@
         <v>62</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D63" s="4" t="s">
         <v>27</v>
@@ -1852,10 +1852,10 @@
         <v>63</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C64" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D64" s="4" t="s">
         <v>33</v>
@@ -1869,10 +1869,10 @@
         <v>64</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C65" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D65" s="4" t="s">
         <v>7</v>
@@ -1886,13 +1886,13 @@
         <v>65</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C66" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="D66" s="4" t="s">
         <v>97</v>
-      </c>
-      <c r="D66" s="4" t="s">
-        <v>98</v>
       </c>
       <c r="E66" s="4">
         <v>4.04</v>
@@ -1903,10 +1903,10 @@
         <v>66</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C67" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D67" s="4" t="s">
         <v>39</v>
@@ -1920,10 +1920,10 @@
         <v>67</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C68" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D68" s="4" t="s">
         <v>5</v>
@@ -1937,10 +1937,10 @@
         <v>68</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C69" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D69" s="4" t="s">
         <v>19</v>
@@ -1954,10 +1954,10 @@
         <v>69</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C70" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D70" s="4" t="s">
         <v>35</v>
@@ -1971,10 +1971,10 @@
         <v>70</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C71" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D71" s="4" t="s">
         <v>13</v>
@@ -1988,10 +1988,10 @@
         <v>71</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C72" s="3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D72" s="4" t="s">
         <v>53</v>
@@ -2005,10 +2005,10 @@
         <v>72</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C73" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D73" s="4" t="s">
         <v>66</v>
@@ -2022,10 +2022,10 @@
         <v>73</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C74" s="3" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D74" s="4" t="s">
         <v>41</v>
@@ -2039,10 +2039,10 @@
         <v>74</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C75" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D75" s="4" t="s">
         <v>13</v>
@@ -2056,10 +2056,10 @@
         <v>75</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C76" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D76" s="4" t="s">
         <v>37</v>

</xml_diff>